<commit_message>
Auto stash before merge of "master" and "origin/master"
</commit_message>
<xml_diff>
--- a/xls2rdf-app/merge_output.xlsx
+++ b/xls2rdf-app/merge_output.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="162">
   <si>
     <t>PREFIX</t>
   </si>
@@ -503,54 +503,6 @@
   </si>
   <si>
     <t>sh:hasValue</t>
-  </si>
-  <si>
-    <t>https://shacl-play.sparna.fr/shapes/Activity</t>
-  </si>
-  <si>
-    <t>sh:NodeShape</t>
-  </si>
-  <si>
-    <t>eli-dl:Activity</t>
-  </si>
-  <si>
-    <t>Activity</t>
-  </si>
-  <si>
-    <t>https://shacl-play.sparna.fr/shapes/Expression</t>
-  </si>
-  <si>
-    <t>eli:Expression</t>
-  </si>
-  <si>
-    <t>Expression</t>
-  </si>
-  <si>
-    <t>https://shacl-play.sparna.fr/shapes/Manifestation</t>
-  </si>
-  <si>
-    <t>eli:Manifestation</t>
-  </si>
-  <si>
-    <t>Manifestation</t>
-  </si>
-  <si>
-    <t>https://shacl-play.sparna.fr/shapes/Work</t>
-  </si>
-  <si>
-    <t>eli:Work</t>
-  </si>
-  <si>
-    <t>Work</t>
-  </si>
-  <si>
-    <t>https://shacl-play.sparna.fr/shapes/WorkSubdivision</t>
-  </si>
-  <si>
-    <t>eli-dl:WorkSubdivision</t>
-  </si>
-  <si>
-    <t>WorkSubdivision</t>
   </si>
 </sst>
 </file>
@@ -1553,76 +1505,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B3" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="7" ht="65" customHeight="1">
-      <c r="A7" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="M7" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="N7" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="O7" s="2"/>
-      <c r="P7" s="2"/>
-    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="s">
         <v>93</v>
@@ -1711,181 +1599,11 @@
         <v>117</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>162</v>
-      </c>
-      <c r="B10" t="s">
-        <v>163</v>
-      </c>
-      <c r="C10" t="s">
-        <v>164</v>
-      </c>
-      <c r="D10" t="s">
-        <v>101</v>
-      </c>
-      <c r="E10" t="s">
-        <v>101</v>
-      </c>
-      <c r="F10" t="s">
-        <v>101</v>
-      </c>
-      <c r="G10" t="s">
-        <v>101</v>
-      </c>
-      <c r="H10" t="s">
-        <v>101</v>
-      </c>
-      <c r="I10" t="s">
-        <v>101</v>
-      </c>
-      <c r="J10" t="s">
-        <v>101</v>
-      </c>
-      <c r="K10" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>166</v>
-      </c>
-      <c r="B11" t="s">
-        <v>163</v>
-      </c>
-      <c r="C11" t="s">
-        <v>167</v>
-      </c>
-      <c r="D11" t="s">
-        <v>101</v>
-      </c>
-      <c r="E11" t="s">
-        <v>101</v>
-      </c>
-      <c r="F11" t="s">
-        <v>101</v>
-      </c>
-      <c r="G11" t="s">
-        <v>101</v>
-      </c>
-      <c r="H11" t="s">
-        <v>101</v>
-      </c>
-      <c r="I11" t="s">
-        <v>101</v>
-      </c>
-      <c r="J11" t="s">
-        <v>101</v>
-      </c>
-      <c r="K11" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>169</v>
-      </c>
-      <c r="B12" t="s">
-        <v>163</v>
-      </c>
-      <c r="C12" t="s">
-        <v>170</v>
-      </c>
-      <c r="D12" t="s">
-        <v>101</v>
-      </c>
-      <c r="E12" t="s">
-        <v>101</v>
-      </c>
-      <c r="F12" t="s">
-        <v>101</v>
-      </c>
-      <c r="G12" t="s">
-        <v>101</v>
-      </c>
-      <c r="H12" t="s">
-        <v>101</v>
-      </c>
-      <c r="I12" t="s">
-        <v>101</v>
-      </c>
-      <c r="J12" t="s">
-        <v>101</v>
-      </c>
-      <c r="K12" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>172</v>
-      </c>
-      <c r="B13" t="s">
-        <v>163</v>
-      </c>
-      <c r="C13" t="s">
-        <v>173</v>
-      </c>
-      <c r="D13" t="s">
-        <v>101</v>
-      </c>
-      <c r="E13" t="s">
-        <v>101</v>
-      </c>
-      <c r="F13" t="s">
-        <v>101</v>
-      </c>
-      <c r="G13" t="s">
-        <v>101</v>
-      </c>
-      <c r="H13" t="s">
-        <v>101</v>
-      </c>
-      <c r="I13" t="s">
-        <v>101</v>
-      </c>
-      <c r="J13" t="s">
-        <v>101</v>
-      </c>
-      <c r="K13" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>175</v>
-      </c>
-      <c r="B14" t="s">
-        <v>163</v>
-      </c>
-      <c r="C14" t="s">
-        <v>176</v>
-      </c>
-      <c r="D14" t="s">
-        <v>101</v>
-      </c>
-      <c r="E14" t="s">
-        <v>101</v>
-      </c>
-      <c r="F14" t="s">
-        <v>101</v>
-      </c>
-      <c r="G14" t="s">
-        <v>101</v>
-      </c>
-      <c r="H14" t="s">
-        <v>101</v>
-      </c>
-      <c r="I14" t="s">
-        <v>101</v>
-      </c>
-      <c r="J14" t="s">
-        <v>101</v>
-      </c>
-      <c r="K14" t="s">
-        <v>177</v>
-      </c>
-    </row>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>